<commit_message>
Deploying to gh-pages from  @ 52f049bc50b483908c70df5e7a954205bcc1f510 🚀
</commit_message>
<xml_diff>
--- a/assets/excel/2026_4-1-5.xlsx
+++ b/assets/excel/2026_4-1-5.xlsx
@@ -8,16 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Hannover\Dez15_Uebergreifende_Analysen\Projekte\Integrationsmonitoring\Schlesier\MT_Site\assets\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{671A7852-E500-4D7D-9B4F-7DE61976659A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D43729AF-4BCB-484D-BE29-F6A5FD35611F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{25B46B2B-FF1A-413B-AD77-D797683F7C16}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId2"/>
-  </externalReferences>
   <calcPr calcId="191029" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -141,7 +138,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="###0.0"/>
+    <numFmt numFmtId="164" formatCode="###0.0"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -405,7 +402,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="3" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="9" fillId="3" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -433,30 +430,6 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -475,6 +448,30 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -493,938 +490,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="2022_4-1-5"/>
-      <sheetName val="2021_Rohdaten"/>
-      <sheetName val="2022_Rohdaten"/>
-      <sheetName val="2023_Rohdaten"/>
-      <sheetName val="2024_Rohdaten"/>
-      <sheetName val="2025_Rohdaten"/>
-      <sheetName val="CSV_Vorbereitung"/>
-      <sheetName val="CSV_Export"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1">
-        <row r="11">
-          <cell r="B11">
-            <v>592.18917499999998</v>
-          </cell>
-          <cell r="C11">
-            <v>4181.3154869999998</v>
-          </cell>
-          <cell r="D11">
-            <v>73.354500000000002</v>
-          </cell>
-          <cell r="E11">
-            <v>785.19937200000004</v>
-          </cell>
-          <cell r="F11">
-            <v>12.387005</v>
-          </cell>
-          <cell r="G11">
-            <v>18.778763999999999</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="B12">
-            <v>302.43057199999998</v>
-          </cell>
-          <cell r="C12">
-            <v>2107.382208</v>
-          </cell>
-          <cell r="D12">
-            <v>42.042909000000002</v>
-          </cell>
-          <cell r="E12">
-            <v>390.46539000000001</v>
-          </cell>
-          <cell r="F12">
-            <v>13.901673000000001</v>
-          </cell>
-          <cell r="G12">
-            <v>18.528455999999998</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="B13">
-            <v>289.75860299999999</v>
-          </cell>
-          <cell r="C13">
-            <v>2073.9332789999999</v>
-          </cell>
-          <cell r="D13">
-            <v>31.311591</v>
-          </cell>
-          <cell r="E13">
-            <v>394.73398200000003</v>
-          </cell>
-          <cell r="F13">
-            <v>10.806094999999999</v>
-          </cell>
-          <cell r="G13">
-            <v>19.033109</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="B14">
-            <v>424.58570900000001</v>
-          </cell>
-          <cell r="C14">
-            <v>3197.6875239999999</v>
-          </cell>
-          <cell r="D14">
-            <v>39.821219999999997</v>
-          </cell>
-          <cell r="E14">
-            <v>420.41152299999999</v>
-          </cell>
-          <cell r="F14">
-            <v>9.3788409999999995</v>
-          </cell>
-          <cell r="G14">
-            <v>13.147361</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="B15">
-            <v>211.81081399999999</v>
-          </cell>
-          <cell r="C15">
-            <v>1599.2633499999999</v>
-          </cell>
-          <cell r="D15">
-            <v>22.064233000000002</v>
-          </cell>
-          <cell r="E15">
-            <v>196.72188600000001</v>
-          </cell>
-          <cell r="F15">
-            <v>10.416952999999999</v>
-          </cell>
-          <cell r="G15">
-            <v>12.300781000000001</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="B16">
-            <v>212.77489499999999</v>
-          </cell>
-          <cell r="C16">
-            <v>1598.424174</v>
-          </cell>
-          <cell r="D16">
-            <v>17.756986999999999</v>
-          </cell>
-          <cell r="E16">
-            <v>223.689637</v>
-          </cell>
-          <cell r="F16">
-            <v>8.3454329999999999</v>
-          </cell>
-          <cell r="G16">
-            <v>13.994384999999999</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="B17">
-            <v>167.603466</v>
-          </cell>
-          <cell r="C17">
-            <v>983.62796300000002</v>
-          </cell>
-          <cell r="D17">
-            <v>33.533279999999998</v>
-          </cell>
-          <cell r="E17">
-            <v>364.78784899999999</v>
-          </cell>
-          <cell r="F17">
-            <v>20.00751</v>
-          </cell>
-          <cell r="G17">
-            <v>37.085957999999998</v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="B18">
-            <v>90.619758000000004</v>
-          </cell>
-          <cell r="C18">
-            <v>508.11885799999999</v>
-          </cell>
-          <cell r="D18">
-            <v>19.978676</v>
-          </cell>
-          <cell r="E18">
-            <v>193.743504</v>
-          </cell>
-          <cell r="F18">
-            <v>22.046710999999998</v>
-          </cell>
-          <cell r="G18">
-            <v>38.129564000000002</v>
-          </cell>
-        </row>
-        <row r="19">
-          <cell r="B19">
-            <v>76.983707999999993</v>
-          </cell>
-          <cell r="C19">
-            <v>475.50910499999998</v>
-          </cell>
-          <cell r="D19">
-            <v>13.554603999999999</v>
-          </cell>
-          <cell r="E19">
-            <v>171.04434499999999</v>
-          </cell>
-          <cell r="F19">
-            <v>17.607106999999999</v>
-          </cell>
-          <cell r="G19">
-            <v>35.970782</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="2">
-        <row r="11">
-          <cell r="B11">
-            <v>598.09607400000004</v>
-          </cell>
-          <cell r="C11">
-            <v>4208.8865130000004</v>
-          </cell>
-          <cell r="D11">
-            <v>78.577333999999993</v>
-          </cell>
-          <cell r="E11">
-            <v>795.09091799999999</v>
-          </cell>
-          <cell r="F11">
-            <v>13.137912</v>
-          </cell>
-          <cell r="G11">
-            <v>18.890765999999999</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="B12">
-            <v>304.02389199999999</v>
-          </cell>
-          <cell r="C12">
-            <v>2111.8473300000001</v>
-          </cell>
-          <cell r="D12">
-            <v>44.418998000000002</v>
-          </cell>
-          <cell r="E12">
-            <v>396.750519</v>
-          </cell>
-          <cell r="F12">
-            <v>14.610364000000001</v>
-          </cell>
-          <cell r="G12">
-            <v>18.786894</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="B13">
-            <v>294.072182</v>
-          </cell>
-          <cell r="C13">
-            <v>2097.0391829999999</v>
-          </cell>
-          <cell r="D13">
-            <v>34.158335999999998</v>
-          </cell>
-          <cell r="E13">
-            <v>398.34039899999999</v>
-          </cell>
-          <cell r="F13">
-            <v>11.615629999999999</v>
-          </cell>
-          <cell r="G13">
-            <v>18.995372</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="B14">
-            <v>425.16594300000003</v>
-          </cell>
-          <cell r="C14">
-            <v>3175.5298630000002</v>
-          </cell>
-          <cell r="D14">
-            <v>41.260734999999997</v>
-          </cell>
-          <cell r="E14">
-            <v>419.421604</v>
-          </cell>
-          <cell r="F14">
-            <v>9.7046189999999992</v>
-          </cell>
-          <cell r="G14">
-            <v>13.207924999999999</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="B15">
-            <v>213.72658000000001</v>
-          </cell>
-          <cell r="C15">
-            <v>1584.246046</v>
-          </cell>
-          <cell r="D15">
-            <v>21.353016</v>
-          </cell>
-          <cell r="E15">
-            <v>198.223061</v>
-          </cell>
-          <cell r="F15">
-            <v>9.9908099999999997</v>
-          </cell>
-          <cell r="G15">
-            <v>12.512138999999999</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="B16">
-            <v>211.43936299999999</v>
-          </cell>
-          <cell r="C16">
-            <v>1591.283817</v>
-          </cell>
-          <cell r="D16">
-            <v>19.907719</v>
-          </cell>
-          <cell r="E16">
-            <v>221.198543</v>
-          </cell>
-          <cell r="F16">
-            <v>9.4153319999999994</v>
-          </cell>
-          <cell r="G16">
-            <v>13.900634</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="B17">
-            <v>172.93013099999999</v>
-          </cell>
-          <cell r="C17">
-            <v>1033.3566499999999</v>
-          </cell>
-          <cell r="D17">
-            <v>37.316598999999997</v>
-          </cell>
-          <cell r="E17">
-            <v>375.66931399999999</v>
-          </cell>
-          <cell r="F17">
-            <v>21.579003</v>
-          </cell>
-          <cell r="G17">
-            <v>36.354275000000001</v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="B18">
-            <v>90.297312000000005</v>
-          </cell>
-          <cell r="C18">
-            <v>527.60128399999996</v>
-          </cell>
-          <cell r="D18">
-            <v>23.065982000000002</v>
-          </cell>
-          <cell r="E18">
-            <v>198.527458</v>
-          </cell>
-          <cell r="F18">
-            <v>25.544484000000001</v>
-          </cell>
-          <cell r="G18">
-            <v>37.628312000000001</v>
-          </cell>
-        </row>
-        <row r="19">
-          <cell r="B19">
-            <v>82.632818999999998</v>
-          </cell>
-          <cell r="C19">
-            <v>505.75536599999998</v>
-          </cell>
-          <cell r="D19">
-            <v>14.250617</v>
-          </cell>
-          <cell r="E19">
-            <v>177.14185599999999</v>
-          </cell>
-          <cell r="F19">
-            <v>17.245711</v>
-          </cell>
-          <cell r="G19">
-            <v>35.025205</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="3">
-        <row r="11">
-          <cell r="B11">
-            <v>593.74429199999997</v>
-          </cell>
-          <cell r="C11">
-            <v>4226.963471</v>
-          </cell>
-          <cell r="D11">
-            <v>85.119185000000002</v>
-          </cell>
-          <cell r="E11">
-            <v>780.83077900000001</v>
-          </cell>
-          <cell r="F11">
-            <v>14.336001</v>
-          </cell>
-          <cell r="G11">
-            <v>18.472617</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="B12">
-            <v>301.280888</v>
-          </cell>
-          <cell r="C12">
-            <v>2120.5386170000002</v>
-          </cell>
-          <cell r="D12">
-            <v>51.275933999999999</v>
-          </cell>
-          <cell r="E12">
-            <v>386.35118699999998</v>
-          </cell>
-          <cell r="F12">
-            <v>17.019311999999999</v>
-          </cell>
-          <cell r="G12">
-            <v>18.219484000000001</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="B13">
-            <v>292.46340400000003</v>
-          </cell>
-          <cell r="C13">
-            <v>2106.4248539999999</v>
-          </cell>
-          <cell r="D13">
-            <v>33.843251000000002</v>
-          </cell>
-          <cell r="E13">
-            <v>394.47959200000003</v>
-          </cell>
-          <cell r="F13">
-            <v>11.57179</v>
-          </cell>
-          <cell r="G13">
-            <v>18.727447000000002</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="B14">
-            <v>404.98306100000002</v>
-          </cell>
-          <cell r="C14">
-            <v>3161.2586980000001</v>
-          </cell>
-          <cell r="D14">
-            <v>41.652287000000001</v>
-          </cell>
-          <cell r="E14">
-            <v>389.62146999999999</v>
-          </cell>
-          <cell r="F14">
-            <v>10.284945</v>
-          </cell>
-          <cell r="G14">
-            <v>12.324884000000001</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="B15">
-            <v>203.14160899999999</v>
-          </cell>
-          <cell r="C15">
-            <v>1579.784566</v>
-          </cell>
-          <cell r="D15">
-            <v>22.880966000000001</v>
-          </cell>
-          <cell r="E15">
-            <v>183.02580800000001</v>
-          </cell>
-          <cell r="F15">
-            <v>11.263555</v>
-          </cell>
-          <cell r="G15">
-            <v>11.585492</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="B16">
-            <v>201.841452</v>
-          </cell>
-          <cell r="C16">
-            <v>1581.4741320000001</v>
-          </cell>
-          <cell r="D16">
-            <v>18.771321</v>
-          </cell>
-          <cell r="E16">
-            <v>206.595662</v>
-          </cell>
-          <cell r="F16">
-            <v>9.3000330000000009</v>
-          </cell>
-          <cell r="G16">
-            <v>13.063487</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="B17">
-            <v>188.76123100000001</v>
-          </cell>
-          <cell r="C17">
-            <v>1065.7047729999999</v>
-          </cell>
-          <cell r="D17">
-            <v>43.466898</v>
-          </cell>
-          <cell r="E17">
-            <v>391.20930900000002</v>
-          </cell>
-          <cell r="F17">
-            <v>23.027450000000002</v>
-          </cell>
-          <cell r="G17">
-            <v>36.708976</v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="B18">
-            <v>98.139279000000002</v>
-          </cell>
-          <cell r="C18">
-            <v>540.754051</v>
-          </cell>
-          <cell r="D18">
-            <v>28.394967999999999</v>
-          </cell>
-          <cell r="E18">
-            <v>203.325379</v>
-          </cell>
-          <cell r="F18">
-            <v>28.933337000000002</v>
-          </cell>
-          <cell r="G18">
-            <v>37.600343000000002</v>
-          </cell>
-        </row>
-        <row r="19">
-          <cell r="B19">
-            <v>90.621951999999993</v>
-          </cell>
-          <cell r="C19">
-            <v>524.95072200000004</v>
-          </cell>
-          <cell r="D19">
-            <v>15.07193</v>
-          </cell>
-          <cell r="E19">
-            <v>187.88392999999999</v>
-          </cell>
-          <cell r="F19">
-            <v>16.631654999999999</v>
-          </cell>
-          <cell r="G19">
-            <v>35.790774999999996</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="4">
-        <row r="11">
-          <cell r="B11">
-            <v>581.27846799999998</v>
-          </cell>
-          <cell r="C11">
-            <v>4225.4592910000001</v>
-          </cell>
-          <cell r="D11">
-            <v>85.762679000000006</v>
-          </cell>
-          <cell r="E11">
-            <v>765.13232900000003</v>
-          </cell>
-          <cell r="F11">
-            <v>14.754147</v>
-          </cell>
-          <cell r="G11">
-            <v>18.107672000000001</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="B12">
-            <v>299.14718699999997</v>
-          </cell>
-          <cell r="C12">
-            <v>2122.7304730000001</v>
-          </cell>
-          <cell r="D12">
-            <v>53.365881000000002</v>
-          </cell>
-          <cell r="E12">
-            <v>382.69006100000001</v>
-          </cell>
-          <cell r="F12">
-            <v>17.839338999999999</v>
-          </cell>
-          <cell r="G12">
-            <v>18.028198</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="B13">
-            <v>282.131281</v>
-          </cell>
-          <cell r="C13">
-            <v>2102.728818</v>
-          </cell>
-          <cell r="D13">
-            <v>32.396797999999997</v>
-          </cell>
-          <cell r="E13">
-            <v>382.44226800000001</v>
-          </cell>
-          <cell r="F13">
-            <v>11.482881000000001</v>
-          </cell>
-          <cell r="G13">
-            <v>18.187902999999999</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="B14">
-            <v>382.071124</v>
-          </cell>
-          <cell r="C14">
-            <v>3079.5796759999998</v>
-          </cell>
-          <cell r="D14">
-            <v>39.997793000000001</v>
-          </cell>
-          <cell r="E14">
-            <v>352.887832</v>
-          </cell>
-          <cell r="F14">
-            <v>10.468677</v>
-          </cell>
-          <cell r="G14">
-            <v>11.458961</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="B15">
-            <v>192.60028299999999</v>
-          </cell>
-          <cell r="C15">
-            <v>1546.9870249999999</v>
-          </cell>
-          <cell r="D15">
-            <v>24.143861999999999</v>
-          </cell>
-          <cell r="E15">
-            <v>167.28674899999999</v>
-          </cell>
-          <cell r="F15">
-            <v>12.535735000000001</v>
-          </cell>
-          <cell r="G15">
-            <v>10.813713999999999</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="B16">
-            <v>189.47084100000001</v>
-          </cell>
-          <cell r="C16">
-            <v>1532.5926509999999</v>
-          </cell>
-          <cell r="D16">
-            <v>15.853930999999999</v>
-          </cell>
-          <cell r="E16">
-            <v>185.60108299999999</v>
-          </cell>
-          <cell r="F16">
-            <v>8.3674780000000002</v>
-          </cell>
-          <cell r="G16">
-            <v>12.110268</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="B17">
-            <v>199.20734400000001</v>
-          </cell>
-          <cell r="C17">
-            <v>1145.8796150000001</v>
-          </cell>
-          <cell r="D17">
-            <v>45.764885999999997</v>
-          </cell>
-          <cell r="E17">
-            <v>412.24449700000002</v>
-          </cell>
-          <cell r="F17">
-            <v>22.973493000000001</v>
-          </cell>
-          <cell r="G17">
-            <v>35.976247999999998</v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="B18">
-            <v>106.546904</v>
-          </cell>
-          <cell r="C18">
-            <v>575.74344799999994</v>
-          </cell>
-          <cell r="D18">
-            <v>29.222019</v>
-          </cell>
-          <cell r="E18">
-            <v>215.403312</v>
-          </cell>
-          <cell r="F18">
-            <v>27.426437</v>
-          </cell>
-          <cell r="G18">
-            <v>37.413072</v>
-          </cell>
-        </row>
-        <row r="19">
-          <cell r="B19">
-            <v>92.660439999999994</v>
-          </cell>
-          <cell r="C19">
-            <v>570.136167</v>
-          </cell>
-          <cell r="D19">
-            <v>16.542867000000001</v>
-          </cell>
-          <cell r="E19">
-            <v>196.841185</v>
-          </cell>
-          <cell r="F19">
-            <v>17.853214000000001</v>
-          </cell>
-          <cell r="G19">
-            <v>34.525292999999998</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="5">
-        <row r="11">
-          <cell r="B11">
-            <v>563.51249499999994</v>
-          </cell>
-          <cell r="C11">
-            <v>4210.8418410000004</v>
-          </cell>
-          <cell r="D11">
-            <v>75.550521000000003</v>
-          </cell>
-          <cell r="E11">
-            <v>650.87234100000001</v>
-          </cell>
-          <cell r="F11">
-            <v>13.407071</v>
-          </cell>
-          <cell r="G11">
-            <v>15.45706</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="B12">
-            <v>291.55767300000002</v>
-          </cell>
-          <cell r="C12">
-            <v>2117.411216</v>
-          </cell>
-          <cell r="D12">
-            <v>44.498083000000001</v>
-          </cell>
-          <cell r="E12">
-            <v>335.08576799999997</v>
-          </cell>
-          <cell r="F12">
-            <v>15.262188999999999</v>
-          </cell>
-          <cell r="G12">
-            <v>15.825257000000001</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="B13">
-            <v>271.95482199999998</v>
-          </cell>
-          <cell r="C13">
-            <v>2093.430625</v>
-          </cell>
-          <cell r="D13">
-            <v>31.052437999999999</v>
-          </cell>
-          <cell r="E13">
-            <v>315.78657299999998</v>
-          </cell>
-          <cell r="F13">
-            <v>11.418234</v>
-          </cell>
-          <cell r="G13">
-            <v>15.084645</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="B14">
-            <v>361.11754500000001</v>
-          </cell>
-          <cell r="C14">
-            <v>3052.163301</v>
-          </cell>
-          <cell r="D14">
-            <v>32.134946999999997</v>
-          </cell>
-          <cell r="E14">
-            <v>259.21451500000001</v>
-          </cell>
-          <cell r="F14">
-            <v>8.8987499999999997</v>
-          </cell>
-          <cell r="G14">
-            <v>8.4928129999999999</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="B15">
-            <v>183.59249</v>
-          </cell>
-          <cell r="C15">
-            <v>1529.4529849999999</v>
-          </cell>
-          <cell r="D15">
-            <v>17.232510999999999</v>
-          </cell>
-          <cell r="E15">
-            <v>123.36502</v>
-          </cell>
-          <cell r="F15">
-            <v>9.3862830000000006</v>
-          </cell>
-          <cell r="G15">
-            <v>8.0659569999999992</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="B16">
-            <v>177.52505500000001</v>
-          </cell>
-          <cell r="C16">
-            <v>1522.7103159999999</v>
-          </cell>
-          <cell r="D16">
-            <v>14.902436</v>
-          </cell>
-          <cell r="E16">
-            <v>135.84949499999999</v>
-          </cell>
-          <cell r="F16">
-            <v>8.3945539999999994</v>
-          </cell>
-          <cell r="G16">
-            <v>8.9215590000000002</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="B17">
-            <v>202.39494999999999</v>
-          </cell>
-          <cell r="C17">
-            <v>1158.6785400000001</v>
-          </cell>
-          <cell r="D17">
-            <v>43.415573999999999</v>
-          </cell>
-          <cell r="E17">
-            <v>391.657826</v>
-          </cell>
-          <cell r="F17">
-            <v>21.450918000000001</v>
-          </cell>
-          <cell r="G17">
-            <v>33.802112999999999</v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="B18">
-            <v>107.965183</v>
-          </cell>
-          <cell r="C18">
-            <v>587.95823099999996</v>
-          </cell>
-          <cell r="D18">
-            <v>27.265571999999999</v>
-          </cell>
-          <cell r="E18">
-            <v>211.72074799999999</v>
-          </cell>
-          <cell r="F18">
-            <v>25.254041000000001</v>
-          </cell>
-          <cell r="G18">
-            <v>36.009487999999997</v>
-          </cell>
-        </row>
-        <row r="19">
-          <cell r="B19">
-            <v>94.429766999999998</v>
-          </cell>
-          <cell r="C19">
-            <v>570.72030900000004</v>
-          </cell>
-          <cell r="D19">
-            <v>16.150002000000001</v>
-          </cell>
-          <cell r="E19">
-            <v>179.93707800000001</v>
-          </cell>
-          <cell r="F19">
-            <v>17.10266</v>
-          </cell>
-          <cell r="G19">
-            <v>31.528065999999999</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1762,40 +827,40 @@
       <c r="D4" s="2"/>
     </row>
     <row r="6" spans="2:10" s="4" customFormat="1" ht="8.25">
-      <c r="B6" s="28" t="s">
+      <c r="B6" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="31" t="s">
+      <c r="C6" s="39" t="s">
         <v>3</v>
       </c>
       <c r="D6" s="3"/>
-      <c r="E6" s="34" t="s">
+      <c r="E6" s="42" t="s">
         <v>4</v>
       </c>
-      <c r="F6" s="34"/>
-      <c r="G6" s="34"/>
-      <c r="H6" s="34"/>
-      <c r="I6" s="34"/>
-      <c r="J6" s="34"/>
+      <c r="F6" s="42"/>
+      <c r="G6" s="42"/>
+      <c r="H6" s="42"/>
+      <c r="I6" s="42"/>
+      <c r="J6" s="42"/>
     </row>
     <row r="7" spans="2:10" s="4" customFormat="1" ht="8.25">
-      <c r="B7" s="29"/>
-      <c r="C7" s="32"/>
+      <c r="B7" s="37"/>
+      <c r="C7" s="40"/>
       <c r="D7" s="5"/>
-      <c r="E7" s="35" t="s">
+      <c r="E7" s="43" t="s">
         <v>5</v>
       </c>
-      <c r="F7" s="35"/>
-      <c r="G7" s="35" t="s">
+      <c r="F7" s="43"/>
+      <c r="G7" s="43" t="s">
         <v>6</v>
       </c>
-      <c r="H7" s="35"/>
-      <c r="I7" s="35"/>
-      <c r="J7" s="35"/>
+      <c r="H7" s="43"/>
+      <c r="I7" s="43"/>
+      <c r="J7" s="43"/>
     </row>
     <row r="8" spans="2:10" s="4" customFormat="1" ht="41.25">
-      <c r="B8" s="29"/>
-      <c r="C8" s="32"/>
+      <c r="B8" s="37"/>
+      <c r="C8" s="40"/>
       <c r="D8" s="5" t="s">
         <v>7</v>
       </c>
@@ -1819,8 +884,8 @@
       </c>
     </row>
     <row r="9" spans="2:10" s="4" customFormat="1" ht="8.25">
-      <c r="B9" s="30"/>
-      <c r="C9" s="33"/>
+      <c r="B9" s="38"/>
+      <c r="C9" s="41"/>
       <c r="D9" s="8"/>
       <c r="E9" s="6" t="s">
         <v>12</v>
@@ -1880,28 +945,22 @@
       <c r="D11" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="36">
-        <f>'[1]2025_Rohdaten'!B11</f>
+      <c r="E11" s="28">
         <v>563.51249499999994</v>
       </c>
-      <c r="F11" s="36">
-        <f>'[1]2025_Rohdaten'!C11</f>
+      <c r="F11" s="28">
         <v>4210.8418410000004</v>
       </c>
-      <c r="G11" s="36">
-        <f>'[1]2025_Rohdaten'!D11</f>
+      <c r="G11" s="28">
         <v>75.550521000000003</v>
       </c>
-      <c r="H11" s="36">
-        <f>'[1]2025_Rohdaten'!E11</f>
+      <c r="H11" s="28">
         <v>650.87234100000001</v>
       </c>
-      <c r="I11" s="36">
-        <f>'[1]2025_Rohdaten'!F11</f>
+      <c r="I11" s="28">
         <v>13.407071</v>
       </c>
-      <c r="J11" s="36">
-        <f>'[1]2025_Rohdaten'!G11</f>
+      <c r="J11" s="28">
         <v>15.45706</v>
       </c>
     </row>
@@ -1915,28 +974,22 @@
       <c r="D12" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="E12" s="36">
-        <f>'[1]2025_Rohdaten'!B12</f>
+      <c r="E12" s="28">
         <v>291.55767300000002</v>
       </c>
-      <c r="F12" s="36">
-        <f>'[1]2025_Rohdaten'!C12</f>
+      <c r="F12" s="28">
         <v>2117.411216</v>
       </c>
-      <c r="G12" s="36">
-        <f>'[1]2025_Rohdaten'!D12</f>
+      <c r="G12" s="28">
         <v>44.498083000000001</v>
       </c>
-      <c r="H12" s="36">
-        <f>'[1]2025_Rohdaten'!E12</f>
+      <c r="H12" s="28">
         <v>335.08576799999997</v>
       </c>
-      <c r="I12" s="36">
-        <f>'[1]2025_Rohdaten'!F12</f>
+      <c r="I12" s="28">
         <v>15.262188999999999</v>
       </c>
-      <c r="J12" s="36">
-        <f>'[1]2025_Rohdaten'!G12</f>
+      <c r="J12" s="28">
         <v>15.825257000000001</v>
       </c>
     </row>
@@ -1950,28 +1003,22 @@
       <c r="D13" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="E13" s="36">
-        <f>'[1]2025_Rohdaten'!B13</f>
+      <c r="E13" s="28">
         <v>271.95482199999998</v>
       </c>
-      <c r="F13" s="36">
-        <f>'[1]2025_Rohdaten'!C13</f>
+      <c r="F13" s="28">
         <v>2093.430625</v>
       </c>
-      <c r="G13" s="36">
-        <f>'[1]2025_Rohdaten'!D13</f>
+      <c r="G13" s="28">
         <v>31.052437999999999</v>
       </c>
-      <c r="H13" s="36">
-        <f>'[1]2025_Rohdaten'!E13</f>
+      <c r="H13" s="28">
         <v>315.78657299999998</v>
       </c>
-      <c r="I13" s="36">
-        <f>'[1]2025_Rohdaten'!F13</f>
+      <c r="I13" s="28">
         <v>11.418234</v>
       </c>
-      <c r="J13" s="36">
-        <f>'[1]2025_Rohdaten'!G13</f>
+      <c r="J13" s="28">
         <v>15.084645</v>
       </c>
     </row>
@@ -1985,28 +1032,22 @@
       <c r="D14" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E14" s="36">
-        <f>'[1]2025_Rohdaten'!B14</f>
+      <c r="E14" s="28">
         <v>361.11754500000001</v>
       </c>
-      <c r="F14" s="36">
-        <f>'[1]2025_Rohdaten'!C14</f>
+      <c r="F14" s="28">
         <v>3052.163301</v>
       </c>
-      <c r="G14" s="36">
-        <f>'[1]2025_Rohdaten'!D14</f>
+      <c r="G14" s="28">
         <v>32.134946999999997</v>
       </c>
-      <c r="H14" s="36">
-        <f>'[1]2025_Rohdaten'!E14</f>
+      <c r="H14" s="28">
         <v>259.21451500000001</v>
       </c>
-      <c r="I14" s="36">
-        <f>'[1]2025_Rohdaten'!F14</f>
+      <c r="I14" s="28">
         <v>8.8987499999999997</v>
       </c>
-      <c r="J14" s="36">
-        <f>'[1]2025_Rohdaten'!G14</f>
+      <c r="J14" s="28">
         <v>8.4928129999999999</v>
       </c>
     </row>
@@ -2020,28 +1061,22 @@
       <c r="D15" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="E15" s="36">
-        <f>'[1]2025_Rohdaten'!B15</f>
+      <c r="E15" s="28">
         <v>183.59249</v>
       </c>
-      <c r="F15" s="36">
-        <f>'[1]2025_Rohdaten'!C15</f>
+      <c r="F15" s="28">
         <v>1529.4529849999999</v>
       </c>
-      <c r="G15" s="36">
-        <f>'[1]2025_Rohdaten'!D15</f>
+      <c r="G15" s="28">
         <v>17.232510999999999</v>
       </c>
-      <c r="H15" s="36">
-        <f>'[1]2025_Rohdaten'!E15</f>
+      <c r="H15" s="28">
         <v>123.36502</v>
       </c>
-      <c r="I15" s="36">
-        <f>'[1]2025_Rohdaten'!F15</f>
+      <c r="I15" s="28">
         <v>9.3862830000000006</v>
       </c>
-      <c r="J15" s="36">
-        <f>'[1]2025_Rohdaten'!G15</f>
+      <c r="J15" s="28">
         <v>8.0659569999999992</v>
       </c>
     </row>
@@ -2055,28 +1090,22 @@
       <c r="D16" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="E16" s="36">
-        <f>'[1]2025_Rohdaten'!B16</f>
+      <c r="E16" s="28">
         <v>177.52505500000001</v>
       </c>
-      <c r="F16" s="36">
-        <f>'[1]2025_Rohdaten'!C16</f>
+      <c r="F16" s="28">
         <v>1522.7103159999999</v>
       </c>
-      <c r="G16" s="36">
-        <f>'[1]2025_Rohdaten'!D16</f>
+      <c r="G16" s="28">
         <v>14.902436</v>
       </c>
-      <c r="H16" s="36">
-        <f>'[1]2025_Rohdaten'!E16</f>
+      <c r="H16" s="28">
         <v>135.84949499999999</v>
       </c>
-      <c r="I16" s="36">
-        <f>'[1]2025_Rohdaten'!F16</f>
+      <c r="I16" s="28">
         <v>8.3945539999999994</v>
       </c>
-      <c r="J16" s="36">
-        <f>'[1]2025_Rohdaten'!G16</f>
+      <c r="J16" s="28">
         <v>8.9215590000000002</v>
       </c>
     </row>
@@ -2090,28 +1119,22 @@
       <c r="D17" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E17" s="36">
-        <f>'[1]2025_Rohdaten'!B17</f>
+      <c r="E17" s="28">
         <v>202.39494999999999</v>
       </c>
-      <c r="F17" s="36">
-        <f>'[1]2025_Rohdaten'!C17</f>
+      <c r="F17" s="28">
         <v>1158.6785400000001</v>
       </c>
-      <c r="G17" s="36">
-        <f>'[1]2025_Rohdaten'!D17</f>
+      <c r="G17" s="28">
         <v>43.415573999999999</v>
       </c>
-      <c r="H17" s="36">
-        <f>'[1]2025_Rohdaten'!E17</f>
+      <c r="H17" s="28">
         <v>391.657826</v>
       </c>
-      <c r="I17" s="36">
-        <f>'[1]2025_Rohdaten'!F17</f>
+      <c r="I17" s="28">
         <v>21.450918000000001</v>
       </c>
-      <c r="J17" s="36">
-        <f>'[1]2025_Rohdaten'!G17</f>
+      <c r="J17" s="28">
         <v>33.802112999999999</v>
       </c>
     </row>
@@ -2125,28 +1148,22 @@
       <c r="D18" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="E18" s="36">
-        <f>'[1]2025_Rohdaten'!B18</f>
+      <c r="E18" s="28">
         <v>107.965183</v>
       </c>
-      <c r="F18" s="36">
-        <f>'[1]2025_Rohdaten'!C18</f>
+      <c r="F18" s="28">
         <v>587.95823099999996</v>
       </c>
-      <c r="G18" s="36">
-        <f>'[1]2025_Rohdaten'!D18</f>
+      <c r="G18" s="28">
         <v>27.265571999999999</v>
       </c>
-      <c r="H18" s="36">
-        <f>'[1]2025_Rohdaten'!E18</f>
+      <c r="H18" s="28">
         <v>211.72074799999999</v>
       </c>
-      <c r="I18" s="36">
-        <f>'[1]2025_Rohdaten'!F18</f>
+      <c r="I18" s="28">
         <v>25.254041000000001</v>
       </c>
-      <c r="J18" s="36">
-        <f>'[1]2025_Rohdaten'!G18</f>
+      <c r="J18" s="28">
         <v>36.009487999999997</v>
       </c>
     </row>
@@ -2160,28 +1177,22 @@
       <c r="D19" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="E19" s="36">
-        <f>'[1]2025_Rohdaten'!B19</f>
+      <c r="E19" s="28">
         <v>94.429766999999998</v>
       </c>
-      <c r="F19" s="36">
-        <f>'[1]2025_Rohdaten'!C19</f>
+      <c r="F19" s="28">
         <v>570.72030900000004</v>
       </c>
-      <c r="G19" s="36">
-        <f>'[1]2025_Rohdaten'!D19</f>
+      <c r="G19" s="28">
         <v>16.150002000000001</v>
       </c>
-      <c r="H19" s="36">
-        <f>'[1]2025_Rohdaten'!E19</f>
+      <c r="H19" s="28">
         <v>179.93707800000001</v>
       </c>
-      <c r="I19" s="36">
-        <f>'[1]2025_Rohdaten'!F19</f>
+      <c r="I19" s="28">
         <v>17.10266</v>
       </c>
-      <c r="J19" s="36">
-        <f>'[1]2025_Rohdaten'!G19</f>
+      <c r="J19" s="28">
         <v>31.528065999999999</v>
       </c>
     </row>
@@ -2195,28 +1206,22 @@
       <c r="D20" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E20" s="36">
-        <f>'[1]2024_Rohdaten'!B11</f>
+      <c r="E20" s="28">
         <v>581.27846799999998</v>
       </c>
-      <c r="F20" s="36">
-        <f>'[1]2024_Rohdaten'!C11</f>
+      <c r="F20" s="28">
         <v>4225.4592910000001</v>
       </c>
-      <c r="G20" s="36">
-        <f>'[1]2024_Rohdaten'!D11</f>
+      <c r="G20" s="28">
         <v>85.762679000000006</v>
       </c>
-      <c r="H20" s="36">
-        <f>'[1]2024_Rohdaten'!E11</f>
+      <c r="H20" s="28">
         <v>765.13232900000003</v>
       </c>
-      <c r="I20" s="36">
-        <f>'[1]2024_Rohdaten'!F11</f>
+      <c r="I20" s="28">
         <v>14.754147</v>
       </c>
-      <c r="J20" s="36">
-        <f>'[1]2024_Rohdaten'!G11</f>
+      <c r="J20" s="28">
         <v>18.107672000000001</v>
       </c>
     </row>
@@ -2230,28 +1235,22 @@
       <c r="D21" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="E21" s="36">
-        <f>'[1]2024_Rohdaten'!B12</f>
+      <c r="E21" s="28">
         <v>299.14718699999997</v>
       </c>
-      <c r="F21" s="36">
-        <f>'[1]2024_Rohdaten'!C12</f>
+      <c r="F21" s="28">
         <v>2122.7304730000001</v>
       </c>
-      <c r="G21" s="36">
-        <f>'[1]2024_Rohdaten'!D12</f>
+      <c r="G21" s="28">
         <v>53.365881000000002</v>
       </c>
-      <c r="H21" s="36">
-        <f>'[1]2024_Rohdaten'!E12</f>
+      <c r="H21" s="28">
         <v>382.69006100000001</v>
       </c>
-      <c r="I21" s="36">
-        <f>'[1]2024_Rohdaten'!F12</f>
+      <c r="I21" s="28">
         <v>17.839338999999999</v>
       </c>
-      <c r="J21" s="36">
-        <f>'[1]2024_Rohdaten'!G12</f>
+      <c r="J21" s="28">
         <v>18.028198</v>
       </c>
     </row>
@@ -2265,28 +1264,22 @@
       <c r="D22" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="E22" s="36">
-        <f>'[1]2024_Rohdaten'!B13</f>
+      <c r="E22" s="28">
         <v>282.131281</v>
       </c>
-      <c r="F22" s="36">
-        <f>'[1]2024_Rohdaten'!C13</f>
+      <c r="F22" s="28">
         <v>2102.728818</v>
       </c>
-      <c r="G22" s="36">
-        <f>'[1]2024_Rohdaten'!D13</f>
+      <c r="G22" s="28">
         <v>32.396797999999997</v>
       </c>
-      <c r="H22" s="36">
-        <f>'[1]2024_Rohdaten'!E13</f>
+      <c r="H22" s="28">
         <v>382.44226800000001</v>
       </c>
-      <c r="I22" s="36">
-        <f>'[1]2024_Rohdaten'!F13</f>
+      <c r="I22" s="28">
         <v>11.482881000000001</v>
       </c>
-      <c r="J22" s="36">
-        <f>'[1]2024_Rohdaten'!G13</f>
+      <c r="J22" s="28">
         <v>18.187902999999999</v>
       </c>
     </row>
@@ -2300,28 +1293,22 @@
       <c r="D23" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E23" s="36">
-        <f>'[1]2024_Rohdaten'!B14</f>
+      <c r="E23" s="28">
         <v>382.071124</v>
       </c>
-      <c r="F23" s="36">
-        <f>'[1]2024_Rohdaten'!C14</f>
+      <c r="F23" s="28">
         <v>3079.5796759999998</v>
       </c>
-      <c r="G23" s="36">
-        <f>'[1]2024_Rohdaten'!D14</f>
+      <c r="G23" s="28">
         <v>39.997793000000001</v>
       </c>
-      <c r="H23" s="36">
-        <f>'[1]2024_Rohdaten'!E14</f>
+      <c r="H23" s="28">
         <v>352.887832</v>
       </c>
-      <c r="I23" s="36">
-        <f>'[1]2024_Rohdaten'!F14</f>
+      <c r="I23" s="28">
         <v>10.468677</v>
       </c>
-      <c r="J23" s="36">
-        <f>'[1]2024_Rohdaten'!G14</f>
+      <c r="J23" s="28">
         <v>11.458961</v>
       </c>
     </row>
@@ -2335,28 +1322,22 @@
       <c r="D24" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="E24" s="36">
-        <f>'[1]2024_Rohdaten'!B15</f>
+      <c r="E24" s="28">
         <v>192.60028299999999</v>
       </c>
-      <c r="F24" s="36">
-        <f>'[1]2024_Rohdaten'!C15</f>
+      <c r="F24" s="28">
         <v>1546.9870249999999</v>
       </c>
-      <c r="G24" s="36">
-        <f>'[1]2024_Rohdaten'!D15</f>
+      <c r="G24" s="28">
         <v>24.143861999999999</v>
       </c>
-      <c r="H24" s="36">
-        <f>'[1]2024_Rohdaten'!E15</f>
+      <c r="H24" s="28">
         <v>167.28674899999999</v>
       </c>
-      <c r="I24" s="36">
-        <f>'[1]2024_Rohdaten'!F15</f>
+      <c r="I24" s="28">
         <v>12.535735000000001</v>
       </c>
-      <c r="J24" s="36">
-        <f>'[1]2024_Rohdaten'!G15</f>
+      <c r="J24" s="28">
         <v>10.813713999999999</v>
       </c>
     </row>
@@ -2370,28 +1351,22 @@
       <c r="D25" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="E25" s="36">
-        <f>'[1]2024_Rohdaten'!B16</f>
+      <c r="E25" s="28">
         <v>189.47084100000001</v>
       </c>
-      <c r="F25" s="36">
-        <f>'[1]2024_Rohdaten'!C16</f>
+      <c r="F25" s="28">
         <v>1532.5926509999999</v>
       </c>
-      <c r="G25" s="36">
-        <f>'[1]2024_Rohdaten'!D16</f>
+      <c r="G25" s="28">
         <v>15.853930999999999</v>
       </c>
-      <c r="H25" s="36">
-        <f>'[1]2024_Rohdaten'!E16</f>
+      <c r="H25" s="28">
         <v>185.60108299999999</v>
       </c>
-      <c r="I25" s="36">
-        <f>'[1]2024_Rohdaten'!F16</f>
+      <c r="I25" s="28">
         <v>8.3674780000000002</v>
       </c>
-      <c r="J25" s="36">
-        <f>'[1]2024_Rohdaten'!G16</f>
+      <c r="J25" s="28">
         <v>12.110268</v>
       </c>
     </row>
@@ -2405,28 +1380,22 @@
       <c r="D26" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E26" s="36">
-        <f>'[1]2024_Rohdaten'!B17</f>
+      <c r="E26" s="28">
         <v>199.20734400000001</v>
       </c>
-      <c r="F26" s="36">
-        <f>'[1]2024_Rohdaten'!C17</f>
+      <c r="F26" s="28">
         <v>1145.8796150000001</v>
       </c>
-      <c r="G26" s="36">
-        <f>'[1]2024_Rohdaten'!D17</f>
+      <c r="G26" s="28">
         <v>45.764885999999997</v>
       </c>
-      <c r="H26" s="36">
-        <f>'[1]2024_Rohdaten'!E17</f>
+      <c r="H26" s="28">
         <v>412.24449700000002</v>
       </c>
-      <c r="I26" s="36">
-        <f>'[1]2024_Rohdaten'!F17</f>
+      <c r="I26" s="28">
         <v>22.973493000000001</v>
       </c>
-      <c r="J26" s="36">
-        <f>'[1]2024_Rohdaten'!G17</f>
+      <c r="J26" s="28">
         <v>35.976247999999998</v>
       </c>
     </row>
@@ -2440,28 +1409,22 @@
       <c r="D27" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="E27" s="36">
-        <f>'[1]2024_Rohdaten'!B18</f>
+      <c r="E27" s="28">
         <v>106.546904</v>
       </c>
-      <c r="F27" s="36">
-        <f>'[1]2024_Rohdaten'!C18</f>
+      <c r="F27" s="28">
         <v>575.74344799999994</v>
       </c>
-      <c r="G27" s="36">
-        <f>'[1]2024_Rohdaten'!D18</f>
+      <c r="G27" s="28">
         <v>29.222019</v>
       </c>
-      <c r="H27" s="36">
-        <f>'[1]2024_Rohdaten'!E18</f>
+      <c r="H27" s="28">
         <v>215.403312</v>
       </c>
-      <c r="I27" s="36">
-        <f>'[1]2024_Rohdaten'!F18</f>
+      <c r="I27" s="28">
         <v>27.426437</v>
       </c>
-      <c r="J27" s="36">
-        <f>'[1]2024_Rohdaten'!G18</f>
+      <c r="J27" s="28">
         <v>37.413072</v>
       </c>
     </row>
@@ -2475,28 +1438,22 @@
       <c r="D28" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="E28" s="36">
-        <f>'[1]2024_Rohdaten'!B19</f>
+      <c r="E28" s="28">
         <v>92.660439999999994</v>
       </c>
-      <c r="F28" s="36">
-        <f>'[1]2024_Rohdaten'!C19</f>
+      <c r="F28" s="28">
         <v>570.136167</v>
       </c>
-      <c r="G28" s="36">
-        <f>'[1]2024_Rohdaten'!D19</f>
+      <c r="G28" s="28">
         <v>16.542867000000001</v>
       </c>
-      <c r="H28" s="36">
-        <f>'[1]2024_Rohdaten'!E19</f>
+      <c r="H28" s="28">
         <v>196.841185</v>
       </c>
-      <c r="I28" s="36">
-        <f>'[1]2024_Rohdaten'!F19</f>
+      <c r="I28" s="28">
         <v>17.853214000000001</v>
       </c>
-      <c r="J28" s="36">
-        <f>'[1]2024_Rohdaten'!G19</f>
+      <c r="J28" s="28">
         <v>34.525292999999998</v>
       </c>
     </row>
@@ -2510,28 +1467,22 @@
       <c r="D29" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E29" s="36">
-        <f>'[1]2023_Rohdaten'!B11</f>
+      <c r="E29" s="28">
         <v>593.74429199999997</v>
       </c>
-      <c r="F29" s="36">
-        <f>'[1]2023_Rohdaten'!C11</f>
+      <c r="F29" s="28">
         <v>4226.963471</v>
       </c>
-      <c r="G29" s="36">
-        <f>'[1]2023_Rohdaten'!D11</f>
+      <c r="G29" s="28">
         <v>85.119185000000002</v>
       </c>
-      <c r="H29" s="36">
-        <f>'[1]2023_Rohdaten'!E11</f>
+      <c r="H29" s="28">
         <v>780.83077900000001</v>
       </c>
-      <c r="I29" s="36">
-        <f>'[1]2023_Rohdaten'!F11</f>
+      <c r="I29" s="28">
         <v>14.336001</v>
       </c>
-      <c r="J29" s="36">
-        <f>'[1]2023_Rohdaten'!G11</f>
+      <c r="J29" s="28">
         <v>18.472617</v>
       </c>
     </row>
@@ -2545,28 +1496,22 @@
       <c r="D30" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="E30" s="36">
-        <f>'[1]2023_Rohdaten'!B12</f>
+      <c r="E30" s="28">
         <v>301.280888</v>
       </c>
-      <c r="F30" s="36">
-        <f>'[1]2023_Rohdaten'!C12</f>
+      <c r="F30" s="28">
         <v>2120.5386170000002</v>
       </c>
-      <c r="G30" s="36">
-        <f>'[1]2023_Rohdaten'!D12</f>
+      <c r="G30" s="28">
         <v>51.275933999999999</v>
       </c>
-      <c r="H30" s="36">
-        <f>'[1]2023_Rohdaten'!E12</f>
+      <c r="H30" s="28">
         <v>386.35118699999998</v>
       </c>
-      <c r="I30" s="36">
-        <f>'[1]2023_Rohdaten'!F12</f>
+      <c r="I30" s="28">
         <v>17.019311999999999</v>
       </c>
-      <c r="J30" s="36">
-        <f>'[1]2023_Rohdaten'!G12</f>
+      <c r="J30" s="28">
         <v>18.219484000000001</v>
       </c>
     </row>
@@ -2580,28 +1525,22 @@
       <c r="D31" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="E31" s="36">
-        <f>'[1]2023_Rohdaten'!B13</f>
+      <c r="E31" s="28">
         <v>292.46340400000003</v>
       </c>
-      <c r="F31" s="36">
-        <f>'[1]2023_Rohdaten'!C13</f>
+      <c r="F31" s="28">
         <v>2106.4248539999999</v>
       </c>
-      <c r="G31" s="36">
-        <f>'[1]2023_Rohdaten'!D13</f>
+      <c r="G31" s="28">
         <v>33.843251000000002</v>
       </c>
-      <c r="H31" s="36">
-        <f>'[1]2023_Rohdaten'!E13</f>
+      <c r="H31" s="28">
         <v>394.47959200000003</v>
       </c>
-      <c r="I31" s="36">
-        <f>'[1]2023_Rohdaten'!F13</f>
+      <c r="I31" s="28">
         <v>11.57179</v>
       </c>
-      <c r="J31" s="36">
-        <f>'[1]2023_Rohdaten'!G13</f>
+      <c r="J31" s="28">
         <v>18.727447000000002</v>
       </c>
     </row>
@@ -2615,28 +1554,22 @@
       <c r="D32" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E32" s="36">
-        <f>'[1]2023_Rohdaten'!B14</f>
+      <c r="E32" s="28">
         <v>404.98306100000002</v>
       </c>
-      <c r="F32" s="36">
-        <f>'[1]2023_Rohdaten'!C14</f>
+      <c r="F32" s="28">
         <v>3161.2586980000001</v>
       </c>
-      <c r="G32" s="36">
-        <f>'[1]2023_Rohdaten'!D14</f>
+      <c r="G32" s="28">
         <v>41.652287000000001</v>
       </c>
-      <c r="H32" s="36">
-        <f>'[1]2023_Rohdaten'!E14</f>
+      <c r="H32" s="28">
         <v>389.62146999999999</v>
       </c>
-      <c r="I32" s="36">
-        <f>'[1]2023_Rohdaten'!F14</f>
+      <c r="I32" s="28">
         <v>10.284945</v>
       </c>
-      <c r="J32" s="36">
-        <f>'[1]2023_Rohdaten'!G14</f>
+      <c r="J32" s="28">
         <v>12.324884000000001</v>
       </c>
     </row>
@@ -2650,28 +1583,22 @@
       <c r="D33" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="E33" s="36">
-        <f>'[1]2023_Rohdaten'!B15</f>
+      <c r="E33" s="28">
         <v>203.14160899999999</v>
       </c>
-      <c r="F33" s="36">
-        <f>'[1]2023_Rohdaten'!C15</f>
+      <c r="F33" s="28">
         <v>1579.784566</v>
       </c>
-      <c r="G33" s="36">
-        <f>'[1]2023_Rohdaten'!D15</f>
+      <c r="G33" s="28">
         <v>22.880966000000001</v>
       </c>
-      <c r="H33" s="36">
-        <f>'[1]2023_Rohdaten'!E15</f>
+      <c r="H33" s="28">
         <v>183.02580800000001</v>
       </c>
-      <c r="I33" s="36">
-        <f>'[1]2023_Rohdaten'!F15</f>
+      <c r="I33" s="28">
         <v>11.263555</v>
       </c>
-      <c r="J33" s="36">
-        <f>'[1]2023_Rohdaten'!G15</f>
+      <c r="J33" s="28">
         <v>11.585492</v>
       </c>
     </row>
@@ -2685,28 +1612,22 @@
       <c r="D34" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="E34" s="36">
-        <f>'[1]2023_Rohdaten'!B16</f>
+      <c r="E34" s="28">
         <v>201.841452</v>
       </c>
-      <c r="F34" s="36">
-        <f>'[1]2023_Rohdaten'!C16</f>
+      <c r="F34" s="28">
         <v>1581.4741320000001</v>
       </c>
-      <c r="G34" s="36">
-        <f>'[1]2023_Rohdaten'!D16</f>
+      <c r="G34" s="28">
         <v>18.771321</v>
       </c>
-      <c r="H34" s="36">
-        <f>'[1]2023_Rohdaten'!E16</f>
+      <c r="H34" s="28">
         <v>206.595662</v>
       </c>
-      <c r="I34" s="36">
-        <f>'[1]2023_Rohdaten'!F16</f>
+      <c r="I34" s="28">
         <v>9.3000330000000009</v>
       </c>
-      <c r="J34" s="36">
-        <f>'[1]2023_Rohdaten'!G16</f>
+      <c r="J34" s="28">
         <v>13.063487</v>
       </c>
     </row>
@@ -2720,28 +1641,22 @@
       <c r="D35" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E35" s="36">
-        <f>'[1]2023_Rohdaten'!B17</f>
+      <c r="E35" s="28">
         <v>188.76123100000001</v>
       </c>
-      <c r="F35" s="36">
-        <f>'[1]2023_Rohdaten'!C17</f>
+      <c r="F35" s="28">
         <v>1065.7047729999999</v>
       </c>
-      <c r="G35" s="36">
-        <f>'[1]2023_Rohdaten'!D17</f>
+      <c r="G35" s="28">
         <v>43.466898</v>
       </c>
-      <c r="H35" s="36">
-        <f>'[1]2023_Rohdaten'!E17</f>
+      <c r="H35" s="28">
         <v>391.20930900000002</v>
       </c>
-      <c r="I35" s="36">
-        <f>'[1]2023_Rohdaten'!F17</f>
+      <c r="I35" s="28">
         <v>23.027450000000002</v>
       </c>
-      <c r="J35" s="36">
-        <f>'[1]2023_Rohdaten'!G17</f>
+      <c r="J35" s="28">
         <v>36.708976</v>
       </c>
     </row>
@@ -2755,28 +1670,22 @@
       <c r="D36" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="E36" s="36">
-        <f>'[1]2023_Rohdaten'!B18</f>
+      <c r="E36" s="28">
         <v>98.139279000000002</v>
       </c>
-      <c r="F36" s="36">
-        <f>'[1]2023_Rohdaten'!C18</f>
+      <c r="F36" s="28">
         <v>540.754051</v>
       </c>
-      <c r="G36" s="36">
-        <f>'[1]2023_Rohdaten'!D18</f>
+      <c r="G36" s="28">
         <v>28.394967999999999</v>
       </c>
-      <c r="H36" s="36">
-        <f>'[1]2023_Rohdaten'!E18</f>
+      <c r="H36" s="28">
         <v>203.325379</v>
       </c>
-      <c r="I36" s="36">
-        <f>'[1]2023_Rohdaten'!F18</f>
+      <c r="I36" s="28">
         <v>28.933337000000002</v>
       </c>
-      <c r="J36" s="36">
-        <f>'[1]2023_Rohdaten'!G18</f>
+      <c r="J36" s="28">
         <v>37.600343000000002</v>
       </c>
     </row>
@@ -2790,28 +1699,22 @@
       <c r="D37" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="E37" s="36">
-        <f>'[1]2023_Rohdaten'!B19</f>
+      <c r="E37" s="28">
         <v>90.621951999999993</v>
       </c>
-      <c r="F37" s="36">
-        <f>'[1]2023_Rohdaten'!C19</f>
+      <c r="F37" s="28">
         <v>524.95072200000004</v>
       </c>
-      <c r="G37" s="36">
-        <f>'[1]2023_Rohdaten'!D19</f>
+      <c r="G37" s="28">
         <v>15.07193</v>
       </c>
-      <c r="H37" s="36">
-        <f>'[1]2023_Rohdaten'!E19</f>
+      <c r="H37" s="28">
         <v>187.88392999999999</v>
       </c>
-      <c r="I37" s="36">
-        <f>'[1]2023_Rohdaten'!F19</f>
+      <c r="I37" s="28">
         <v>16.631654999999999</v>
       </c>
-      <c r="J37" s="36">
-        <f>'[1]2023_Rohdaten'!G19</f>
+      <c r="J37" s="28">
         <v>35.790774999999996</v>
       </c>
     </row>
@@ -2825,28 +1728,22 @@
       <c r="D38" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E38" s="36">
-        <f>'[1]2022_Rohdaten'!B11</f>
+      <c r="E38" s="28">
         <v>598.09607400000004</v>
       </c>
-      <c r="F38" s="36">
-        <f>'[1]2022_Rohdaten'!C11</f>
+      <c r="F38" s="28">
         <v>4208.8865130000004</v>
       </c>
-      <c r="G38" s="36">
-        <f>'[1]2022_Rohdaten'!D11</f>
+      <c r="G38" s="28">
         <v>78.577333999999993</v>
       </c>
-      <c r="H38" s="36">
-        <f>'[1]2022_Rohdaten'!E11</f>
+      <c r="H38" s="28">
         <v>795.09091799999999</v>
       </c>
       <c r="I38" s="27">
-        <f>'[1]2022_Rohdaten'!F11</f>
         <v>13.137912</v>
       </c>
       <c r="J38" s="27">
-        <f>'[1]2022_Rohdaten'!G11</f>
         <v>18.890765999999999</v>
       </c>
     </row>
@@ -2860,28 +1757,22 @@
       <c r="D39" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="E39" s="36">
-        <f>'[1]2022_Rohdaten'!B12</f>
+      <c r="E39" s="28">
         <v>304.02389199999999</v>
       </c>
-      <c r="F39" s="36">
-        <f>'[1]2022_Rohdaten'!C12</f>
+      <c r="F39" s="28">
         <v>2111.8473300000001</v>
       </c>
-      <c r="G39" s="36">
-        <f>'[1]2022_Rohdaten'!D12</f>
+      <c r="G39" s="28">
         <v>44.418998000000002</v>
       </c>
-      <c r="H39" s="36">
-        <f>'[1]2022_Rohdaten'!E12</f>
+      <c r="H39" s="28">
         <v>396.750519</v>
       </c>
       <c r="I39" s="27">
-        <f>'[1]2022_Rohdaten'!F12</f>
         <v>14.610364000000001</v>
       </c>
       <c r="J39" s="27">
-        <f>'[1]2022_Rohdaten'!G12</f>
         <v>18.786894</v>
       </c>
     </row>
@@ -2895,28 +1786,22 @@
       <c r="D40" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="E40" s="36">
-        <f>'[1]2022_Rohdaten'!B13</f>
+      <c r="E40" s="28">
         <v>294.072182</v>
       </c>
-      <c r="F40" s="36">
-        <f>'[1]2022_Rohdaten'!C13</f>
+      <c r="F40" s="28">
         <v>2097.0391829999999</v>
       </c>
-      <c r="G40" s="36">
-        <f>'[1]2022_Rohdaten'!D13</f>
+      <c r="G40" s="28">
         <v>34.158335999999998</v>
       </c>
-      <c r="H40" s="36">
-        <f>'[1]2022_Rohdaten'!E13</f>
+      <c r="H40" s="28">
         <v>398.34039899999999</v>
       </c>
       <c r="I40" s="27">
-        <f>'[1]2022_Rohdaten'!F13</f>
         <v>11.615629999999999</v>
       </c>
       <c r="J40" s="27">
-        <f>'[1]2022_Rohdaten'!G13</f>
         <v>18.995372</v>
       </c>
     </row>
@@ -2930,28 +1815,22 @@
       <c r="D41" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E41" s="36">
-        <f>'[1]2022_Rohdaten'!B14</f>
+      <c r="E41" s="28">
         <v>425.16594300000003</v>
       </c>
-      <c r="F41" s="36">
-        <f>'[1]2022_Rohdaten'!C14</f>
+      <c r="F41" s="28">
         <v>3175.5298630000002</v>
       </c>
-      <c r="G41" s="36">
-        <f>'[1]2022_Rohdaten'!D14</f>
+      <c r="G41" s="28">
         <v>41.260734999999997</v>
       </c>
-      <c r="H41" s="36">
-        <f>'[1]2022_Rohdaten'!E14</f>
+      <c r="H41" s="28">
         <v>419.421604</v>
       </c>
       <c r="I41" s="27">
-        <f>'[1]2022_Rohdaten'!F14</f>
         <v>9.7046189999999992</v>
       </c>
       <c r="J41" s="27">
-        <f>'[1]2022_Rohdaten'!G14</f>
         <v>13.207924999999999</v>
       </c>
     </row>
@@ -2965,28 +1844,22 @@
       <c r="D42" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="E42" s="36">
-        <f>'[1]2022_Rohdaten'!B15</f>
+      <c r="E42" s="28">
         <v>213.72658000000001</v>
       </c>
-      <c r="F42" s="36">
-        <f>'[1]2022_Rohdaten'!C15</f>
+      <c r="F42" s="28">
         <v>1584.246046</v>
       </c>
-      <c r="G42" s="36">
-        <f>'[1]2022_Rohdaten'!D15</f>
+      <c r="G42" s="28">
         <v>21.353016</v>
       </c>
-      <c r="H42" s="36">
-        <f>'[1]2022_Rohdaten'!E15</f>
+      <c r="H42" s="28">
         <v>198.223061</v>
       </c>
       <c r="I42" s="27">
-        <f>'[1]2022_Rohdaten'!F15</f>
         <v>9.9908099999999997</v>
       </c>
       <c r="J42" s="27">
-        <f>'[1]2022_Rohdaten'!G15</f>
         <v>12.512138999999999</v>
       </c>
     </row>
@@ -3000,28 +1873,22 @@
       <c r="D43" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="E43" s="36">
-        <f>'[1]2022_Rohdaten'!B16</f>
+      <c r="E43" s="28">
         <v>211.43936299999999</v>
       </c>
-      <c r="F43" s="36">
-        <f>'[1]2022_Rohdaten'!C16</f>
+      <c r="F43" s="28">
         <v>1591.283817</v>
       </c>
-      <c r="G43" s="36">
-        <f>'[1]2022_Rohdaten'!D16</f>
+      <c r="G43" s="28">
         <v>19.907719</v>
       </c>
-      <c r="H43" s="36">
-        <f>'[1]2022_Rohdaten'!E16</f>
+      <c r="H43" s="28">
         <v>221.198543</v>
       </c>
       <c r="I43" s="27">
-        <f>'[1]2022_Rohdaten'!F16</f>
         <v>9.4153319999999994</v>
       </c>
       <c r="J43" s="27">
-        <f>'[1]2022_Rohdaten'!G16</f>
         <v>13.900634</v>
       </c>
     </row>
@@ -3035,28 +1902,22 @@
       <c r="D44" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E44" s="36">
-        <f>'[1]2022_Rohdaten'!B17</f>
+      <c r="E44" s="28">
         <v>172.93013099999999</v>
       </c>
-      <c r="F44" s="36">
-        <f>'[1]2022_Rohdaten'!C17</f>
+      <c r="F44" s="28">
         <v>1033.3566499999999</v>
       </c>
-      <c r="G44" s="36">
-        <f>'[1]2022_Rohdaten'!D17</f>
+      <c r="G44" s="28">
         <v>37.316598999999997</v>
       </c>
-      <c r="H44" s="36">
-        <f>'[1]2022_Rohdaten'!E17</f>
+      <c r="H44" s="28">
         <v>375.66931399999999</v>
       </c>
       <c r="I44" s="27">
-        <f>'[1]2022_Rohdaten'!F17</f>
         <v>21.579003</v>
       </c>
       <c r="J44" s="27">
-        <f>'[1]2022_Rohdaten'!G17</f>
         <v>36.354275000000001</v>
       </c>
     </row>
@@ -3070,28 +1931,22 @@
       <c r="D45" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="E45" s="36">
-        <f>'[1]2022_Rohdaten'!B18</f>
+      <c r="E45" s="28">
         <v>90.297312000000005</v>
       </c>
-      <c r="F45" s="36">
-        <f>'[1]2022_Rohdaten'!C18</f>
+      <c r="F45" s="28">
         <v>527.60128399999996</v>
       </c>
-      <c r="G45" s="36">
-        <f>'[1]2022_Rohdaten'!D18</f>
+      <c r="G45" s="28">
         <v>23.065982000000002</v>
       </c>
-      <c r="H45" s="36">
-        <f>'[1]2022_Rohdaten'!E18</f>
+      <c r="H45" s="28">
         <v>198.527458</v>
       </c>
       <c r="I45" s="27">
-        <f>'[1]2022_Rohdaten'!F18</f>
         <v>25.544484000000001</v>
       </c>
       <c r="J45" s="27">
-        <f>'[1]2022_Rohdaten'!G18</f>
         <v>37.628312000000001</v>
       </c>
     </row>
@@ -3105,32 +1960,26 @@
       <c r="D46" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="E46" s="36">
-        <f>'[1]2022_Rohdaten'!B19</f>
+      <c r="E46" s="28">
         <v>82.632818999999998</v>
       </c>
-      <c r="F46" s="36">
-        <f>'[1]2022_Rohdaten'!C19</f>
+      <c r="F46" s="28">
         <v>505.75536599999998</v>
       </c>
-      <c r="G46" s="36">
-        <f>'[1]2022_Rohdaten'!D19</f>
+      <c r="G46" s="28">
         <v>14.250617</v>
       </c>
-      <c r="H46" s="36">
-        <f>'[1]2022_Rohdaten'!E19</f>
+      <c r="H46" s="28">
         <v>177.14185599999999</v>
       </c>
       <c r="I46" s="27">
-        <f>'[1]2022_Rohdaten'!F19</f>
         <v>17.245711</v>
       </c>
       <c r="J46" s="27">
-        <f>'[1]2022_Rohdaten'!G19</f>
         <v>35.025205</v>
       </c>
     </row>
-    <row r="47" spans="2:10" s="37" customFormat="1" ht="8.25" customHeight="1">
+    <row r="47" spans="2:10" s="29" customFormat="1" ht="8.25" customHeight="1">
       <c r="B47" s="26">
         <v>2021</v>
       </c>
@@ -3140,32 +1989,26 @@
       <c r="D47" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E47" s="36">
-        <f>'[1]2021_Rohdaten'!B11</f>
+      <c r="E47" s="28">
         <v>592.18917499999998</v>
       </c>
-      <c r="F47" s="36">
-        <f>'[1]2021_Rohdaten'!C11</f>
+      <c r="F47" s="28">
         <v>4181.3154869999998</v>
       </c>
-      <c r="G47" s="36">
-        <f>'[1]2021_Rohdaten'!D11</f>
+      <c r="G47" s="28">
         <v>73.354500000000002</v>
       </c>
-      <c r="H47" s="36">
-        <f>'[1]2021_Rohdaten'!E11</f>
+      <c r="H47" s="28">
         <v>785.19937200000004</v>
       </c>
       <c r="I47" s="27">
-        <f>'[1]2021_Rohdaten'!F11</f>
         <v>12.387005</v>
       </c>
       <c r="J47" s="27">
-        <f>'[1]2021_Rohdaten'!G11</f>
         <v>18.778763999999999</v>
       </c>
     </row>
-    <row r="48" spans="2:10" s="37" customFormat="1" ht="8.25" customHeight="1">
+    <row r="48" spans="2:10" s="29" customFormat="1" ht="8.25" customHeight="1">
       <c r="B48" s="26">
         <v>2021</v>
       </c>
@@ -3175,32 +2018,26 @@
       <c r="D48" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="E48" s="36">
-        <f>'[1]2021_Rohdaten'!B12</f>
+      <c r="E48" s="28">
         <v>302.43057199999998</v>
       </c>
-      <c r="F48" s="36">
-        <f>'[1]2021_Rohdaten'!C12</f>
+      <c r="F48" s="28">
         <v>2107.382208</v>
       </c>
-      <c r="G48" s="36">
-        <f>'[1]2021_Rohdaten'!D12</f>
+      <c r="G48" s="28">
         <v>42.042909000000002</v>
       </c>
-      <c r="H48" s="36">
-        <f>'[1]2021_Rohdaten'!E12</f>
+      <c r="H48" s="28">
         <v>390.46539000000001</v>
       </c>
       <c r="I48" s="27">
-        <f>'[1]2021_Rohdaten'!F12</f>
         <v>13.901673000000001</v>
       </c>
       <c r="J48" s="27">
-        <f>'[1]2021_Rohdaten'!G12</f>
         <v>18.528455999999998</v>
       </c>
     </row>
-    <row r="49" spans="1:13" s="38" customFormat="1" ht="8.25" customHeight="1">
+    <row r="49" spans="1:13" s="30" customFormat="1" ht="8.25" customHeight="1">
       <c r="B49" s="26">
         <v>2021</v>
       </c>
@@ -3210,34 +2047,28 @@
       <c r="D49" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="E49" s="36">
-        <f>'[1]2021_Rohdaten'!B13</f>
+      <c r="E49" s="28">
         <v>289.75860299999999</v>
       </c>
-      <c r="F49" s="36">
-        <f>'[1]2021_Rohdaten'!C13</f>
+      <c r="F49" s="28">
         <v>2073.9332789999999</v>
       </c>
-      <c r="G49" s="36">
-        <f>'[1]2021_Rohdaten'!D13</f>
+      <c r="G49" s="28">
         <v>31.311591</v>
       </c>
-      <c r="H49" s="36">
-        <f>'[1]2021_Rohdaten'!E13</f>
+      <c r="H49" s="28">
         <v>394.73398200000003</v>
       </c>
       <c r="I49" s="27">
-        <f>'[1]2021_Rohdaten'!F13</f>
         <v>10.806094999999999</v>
       </c>
       <c r="J49" s="27">
-        <f>'[1]2021_Rohdaten'!G13</f>
         <v>19.033109</v>
       </c>
-      <c r="K49" s="39"/>
-      <c r="L49" s="39"/>
-    </row>
-    <row r="50" spans="1:13" s="38" customFormat="1" ht="8.25" customHeight="1">
+      <c r="K49" s="31"/>
+      <c r="L49" s="31"/>
+    </row>
+    <row r="50" spans="1:13" s="30" customFormat="1" ht="8.25" customHeight="1">
       <c r="B50" s="26">
         <v>2021</v>
       </c>
@@ -3247,34 +2078,28 @@
       <c r="D50" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E50" s="36">
-        <f>'[1]2021_Rohdaten'!B14</f>
+      <c r="E50" s="28">
         <v>424.58570900000001</v>
       </c>
-      <c r="F50" s="36">
-        <f>'[1]2021_Rohdaten'!C14</f>
+      <c r="F50" s="28">
         <v>3197.6875239999999</v>
       </c>
-      <c r="G50" s="36">
-        <f>'[1]2021_Rohdaten'!D14</f>
+      <c r="G50" s="28">
         <v>39.821219999999997</v>
       </c>
-      <c r="H50" s="36">
-        <f>'[1]2021_Rohdaten'!E14</f>
+      <c r="H50" s="28">
         <v>420.41152299999999</v>
       </c>
       <c r="I50" s="27">
-        <f>'[1]2021_Rohdaten'!F14</f>
         <v>9.3788409999999995</v>
       </c>
       <c r="J50" s="27">
-        <f>'[1]2021_Rohdaten'!G14</f>
         <v>13.147361</v>
       </c>
-      <c r="K50" s="40"/>
-      <c r="L50" s="40"/>
-    </row>
-    <row r="51" spans="1:13" s="38" customFormat="1" ht="8.25" customHeight="1">
+      <c r="K50" s="32"/>
+      <c r="L50" s="32"/>
+    </row>
+    <row r="51" spans="1:13" s="30" customFormat="1" ht="8.25" customHeight="1">
       <c r="B51" s="26">
         <v>2021</v>
       </c>
@@ -3284,35 +2109,29 @@
       <c r="D51" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="E51" s="36">
-        <f>'[1]2021_Rohdaten'!B15</f>
+      <c r="E51" s="28">
         <v>211.81081399999999</v>
       </c>
-      <c r="F51" s="36">
-        <f>'[1]2021_Rohdaten'!C15</f>
+      <c r="F51" s="28">
         <v>1599.2633499999999</v>
       </c>
-      <c r="G51" s="36">
-        <f>'[1]2021_Rohdaten'!D15</f>
+      <c r="G51" s="28">
         <v>22.064233000000002</v>
       </c>
-      <c r="H51" s="36">
-        <f>'[1]2021_Rohdaten'!E15</f>
+      <c r="H51" s="28">
         <v>196.72188600000001</v>
       </c>
       <c r="I51" s="27">
-        <f>'[1]2021_Rohdaten'!F15</f>
         <v>10.416952999999999</v>
       </c>
       <c r="J51" s="27">
-        <f>'[1]2021_Rohdaten'!G15</f>
         <v>12.300781000000001</v>
       </c>
-      <c r="K51" s="41"/>
-      <c r="L51" s="41"/>
-    </row>
-    <row r="52" spans="1:13" s="43" customFormat="1" ht="8.25" customHeight="1">
-      <c r="A52" s="42"/>
+      <c r="K51" s="33"/>
+      <c r="L51" s="33"/>
+    </row>
+    <row r="52" spans="1:13" s="35" customFormat="1" ht="8.25" customHeight="1">
+      <c r="A52" s="34"/>
       <c r="B52" s="26">
         <v>2021</v>
       </c>
@@ -3322,35 +2141,29 @@
       <c r="D52" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="E52" s="36">
-        <f>'[1]2021_Rohdaten'!B16</f>
+      <c r="E52" s="28">
         <v>212.77489499999999</v>
       </c>
-      <c r="F52" s="36">
-        <f>'[1]2021_Rohdaten'!C16</f>
+      <c r="F52" s="28">
         <v>1598.424174</v>
       </c>
-      <c r="G52" s="36">
-        <f>'[1]2021_Rohdaten'!D16</f>
+      <c r="G52" s="28">
         <v>17.756986999999999</v>
       </c>
-      <c r="H52" s="36">
-        <f>'[1]2021_Rohdaten'!E16</f>
+      <c r="H52" s="28">
         <v>223.689637</v>
       </c>
       <c r="I52" s="27">
-        <f>'[1]2021_Rohdaten'!F16</f>
         <v>8.3454329999999999</v>
       </c>
       <c r="J52" s="27">
-        <f>'[1]2021_Rohdaten'!G16</f>
         <v>13.994384999999999</v>
       </c>
-      <c r="K52" s="42"/>
-      <c r="L52" s="42"/>
-      <c r="M52" s="42"/>
-    </row>
-    <row r="53" spans="1:13" s="43" customFormat="1" ht="8.25" customHeight="1">
+      <c r="K52" s="34"/>
+      <c r="L52" s="34"/>
+      <c r="M52" s="34"/>
+    </row>
+    <row r="53" spans="1:13" s="35" customFormat="1" ht="8.25" customHeight="1">
       <c r="B53" s="26">
         <v>2021</v>
       </c>
@@ -3360,32 +2173,26 @@
       <c r="D53" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E53" s="36">
-        <f>'[1]2021_Rohdaten'!B17</f>
+      <c r="E53" s="28">
         <v>167.603466</v>
       </c>
-      <c r="F53" s="36">
-        <f>'[1]2021_Rohdaten'!C17</f>
+      <c r="F53" s="28">
         <v>983.62796300000002</v>
       </c>
-      <c r="G53" s="36">
-        <f>'[1]2021_Rohdaten'!D17</f>
+      <c r="G53" s="28">
         <v>33.533279999999998</v>
       </c>
-      <c r="H53" s="36">
-        <f>'[1]2021_Rohdaten'!E17</f>
+      <c r="H53" s="28">
         <v>364.78784899999999</v>
       </c>
       <c r="I53" s="27">
-        <f>'[1]2021_Rohdaten'!F17</f>
         <v>20.00751</v>
       </c>
       <c r="J53" s="27">
-        <f>'[1]2021_Rohdaten'!G17</f>
         <v>37.085957999999998</v>
       </c>
     </row>
-    <row r="54" spans="1:13" s="37" customFormat="1" ht="8.25" customHeight="1">
+    <row r="54" spans="1:13" s="29" customFormat="1" ht="8.25" customHeight="1">
       <c r="B54" s="26">
         <v>2021</v>
       </c>
@@ -3395,32 +2202,26 @@
       <c r="D54" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="E54" s="36">
-        <f>'[1]2021_Rohdaten'!B18</f>
+      <c r="E54" s="28">
         <v>90.619758000000004</v>
       </c>
-      <c r="F54" s="36">
-        <f>'[1]2021_Rohdaten'!C18</f>
+      <c r="F54" s="28">
         <v>508.11885799999999</v>
       </c>
-      <c r="G54" s="36">
-        <f>'[1]2021_Rohdaten'!D18</f>
+      <c r="G54" s="28">
         <v>19.978676</v>
       </c>
-      <c r="H54" s="36">
-        <f>'[1]2021_Rohdaten'!E18</f>
+      <c r="H54" s="28">
         <v>193.743504</v>
       </c>
       <c r="I54" s="27">
-        <f>'[1]2021_Rohdaten'!F18</f>
         <v>22.046710999999998</v>
       </c>
       <c r="J54" s="27">
-        <f>'[1]2021_Rohdaten'!G18</f>
         <v>38.129564000000002</v>
       </c>
     </row>
-    <row r="55" spans="1:13" s="37" customFormat="1" ht="8.25" customHeight="1">
+    <row r="55" spans="1:13" s="29" customFormat="1" ht="8.25" customHeight="1">
       <c r="B55" s="26">
         <v>2021</v>
       </c>
@@ -3430,28 +2231,22 @@
       <c r="D55" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="E55" s="36">
-        <f>'[1]2021_Rohdaten'!B19</f>
+      <c r="E55" s="28">
         <v>76.983707999999993</v>
       </c>
-      <c r="F55" s="36">
-        <f>'[1]2021_Rohdaten'!C19</f>
+      <c r="F55" s="28">
         <v>475.50910499999998</v>
       </c>
-      <c r="G55" s="36">
-        <f>'[1]2021_Rohdaten'!D19</f>
+      <c r="G55" s="28">
         <v>13.554603999999999</v>
       </c>
-      <c r="H55" s="36">
-        <f>'[1]2021_Rohdaten'!E19</f>
+      <c r="H55" s="28">
         <v>171.04434499999999</v>
       </c>
       <c r="I55" s="27">
-        <f>'[1]2021_Rohdaten'!F19</f>
         <v>17.607106999999999</v>
       </c>
       <c r="J55" s="27">
-        <f>'[1]2021_Rohdaten'!G19</f>
         <v>35.970782</v>
       </c>
     </row>

</xml_diff>

<commit_message>
FN Korrektur DL Tabelle
</commit_message>
<xml_diff>
--- a/assets/excel/2026_4-1-5.xlsx
+++ b/assets/excel/2026_4-1-5.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Hannover\Dez15_Uebergreifende_Analysen\Projekte\Integrationsmonitoring\Schlesier\MT_Site\assets\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BiesterChristophLSN\Desktop\MZ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D43729AF-4BCB-484D-BE29-F6A5FD35611F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{81A6BD7D-24BF-4F2A-B887-24FB8A233B22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{25B46B2B-FF1A-413B-AD77-D797683F7C16}"/>
+    <workbookView xWindow="20052" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{25B46B2B-FF1A-413B-AD77-D797683F7C16}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="33">
   <si>
     <t>Indikator 4.1.5: Frühe Schulabgänger/-innen und Personen mit niedrigem Bildungsstand nach Migrationsstatus und Geschlecht</t>
   </si>
@@ -131,6 +131,18 @@
   </si>
   <si>
     <t>Migration und Teilhabe - Integrationsmonitoring Niedersachsen 2026</t>
+  </si>
+  <si>
+    <t>https://www.destatis.de/DE/Themen/Gesellschaft-Umwelt/Bevoelkerung/Haushalte-Familien/Methoden/mikrozensus-2020.html</t>
+  </si>
+  <si>
+    <t>3)  Ab der Veröffentlichung der Endergebnisse 2023 und der Erstergebnisse 2024 werden für die Hochrechnung des Mikrozensus Daten der Bevölkerungsfortschreibung herangezogen, die auf den Eckwerten des Zensus 2022 basieren. Die Hochrechnung für die Jahre vor 2011 sowie für bislang veröffentlichte Ergebnisse des Mikrozensus 2011-2013 basiert auf den fortgeschriebenen Ergebnissen der Volkszählung 1987. In 2016 erfolgte die Umstellung auf eine neue Mikrozensus-Stichprobe (auf Basis des Zensus 2011). Ab 2017 wird nur noch die Bevölkerung in Privathaushalten (ohne Gemeinschaftsunterkünfte) ausgewiesen. Dadurch ergibt sich jeweils eine eingeschränkte Vergleichbarkeit mit den Vorjahren.</t>
+  </si>
+  <si>
+    <t>4) Seit dem Jahr 2018 wird im Mikrozensus der Migrationshintergrund im weiteren Sinne jährlich berichtet. Die in der Tabelle ab dem Jahr 2018 abgebildeten Daten zum Migrationshintergrund entsprechen dem Migrationshintergrund im weiteren Sinne, bis 2017 wird der Migrationshintergrund im engeren Sinne abgebildet. Die Vergleichbarkeit ist dadurch eingeschränkt.</t>
+  </si>
+  <si>
+    <t>5) Die Ergebnisse des Mikrozensus 2020 sind unter anderem aufgrund methodischer Effekte im Rahmen einer Neugestaltung der Erhebung sowie insbesondere aufgrund der Folgen der Corona-Pandemie in Ihrer Datenqualität eingeschränkt. Auf die Verwendung dieser Ergebnisse wird daher verzichtet. Weitere Informationen zur methodischen Neugestaltung des Mikrozensus ab 2020 und zu den Auswirkungen der Neugestaltung und der Corona-Krise auf die Ergebnisse des Jahres 2020 finden Sie auf der Informationsseite des Statistischen Bundesamtes:</t>
   </si>
 </sst>
 </file>
@@ -362,7 +374,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
@@ -471,6 +483,15 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -493,9 +514,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -533,7 +554,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -639,7 +660,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -781,7 +802,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -790,7 +811,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D08CA7DC-4AB7-41CE-9601-7AD578505D24}">
   <sheetPr codeName="Tabelle1"/>
-  <dimension ref="A1:M67"/>
+  <dimension ref="A1:M72"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.85546875" customWidth="1"/>
@@ -2301,65 +2322,145 @@
       <c r="K60" s="18"/>
       <c r="L60" s="18"/>
     </row>
-    <row r="61" spans="1:13" s="21" customFormat="1" ht="8.25" customHeight="1">
-      <c r="A61" s="19"/>
-      <c r="B61" s="20"/>
-      <c r="C61" s="20"/>
-      <c r="D61" s="20"/>
-      <c r="E61" s="20"/>
-      <c r="F61" s="20"/>
-      <c r="G61" s="20"/>
-      <c r="H61" s="20"/>
-      <c r="I61" s="20"/>
-      <c r="J61" s="20"/>
-      <c r="K61" s="19"/>
-      <c r="L61" s="19"/>
-      <c r="M61" s="19"/>
-    </row>
-    <row r="62" spans="1:13" s="21" customFormat="1" ht="8.25" customHeight="1">
-      <c r="B62" s="22" t="s">
+    <row r="61" spans="1:13" s="13" customFormat="1" ht="26.25" customHeight="1">
+      <c r="B61" s="44" t="s">
+        <v>30</v>
+      </c>
+      <c r="C61" s="44"/>
+      <c r="D61" s="44"/>
+      <c r="E61" s="44"/>
+      <c r="F61" s="44"/>
+      <c r="G61" s="44"/>
+      <c r="H61" s="44"/>
+      <c r="I61" s="44"/>
+      <c r="J61" s="44"/>
+      <c r="K61" s="44"/>
+      <c r="L61" s="44"/>
+      <c r="M61" s="44"/>
+    </row>
+    <row r="62" spans="1:13" s="13" customFormat="1" ht="20.25" customHeight="1">
+      <c r="B62" s="44" t="s">
+        <v>31</v>
+      </c>
+      <c r="C62" s="44"/>
+      <c r="D62" s="44"/>
+      <c r="E62" s="44"/>
+      <c r="F62" s="44"/>
+      <c r="G62" s="44"/>
+      <c r="H62" s="44"/>
+      <c r="I62" s="44"/>
+      <c r="J62" s="44"/>
+      <c r="K62" s="44"/>
+      <c r="L62" s="44"/>
+      <c r="M62" s="44"/>
+    </row>
+    <row r="63" spans="1:13" s="13" customFormat="1" ht="24" customHeight="1">
+      <c r="B63" s="44" t="s">
+        <v>32</v>
+      </c>
+      <c r="C63" s="44"/>
+      <c r="D63" s="44"/>
+      <c r="E63" s="44"/>
+      <c r="F63" s="44"/>
+      <c r="G63" s="44"/>
+      <c r="H63" s="44"/>
+      <c r="I63" s="44"/>
+      <c r="J63" s="44"/>
+      <c r="K63" s="44"/>
+      <c r="L63" s="44"/>
+      <c r="M63" s="44"/>
+    </row>
+    <row r="64" spans="1:13" s="13" customFormat="1" ht="8.25" customHeight="1">
+      <c r="B64" s="45" t="s">
+        <v>29</v>
+      </c>
+      <c r="C64" s="46"/>
+      <c r="D64" s="46"/>
+      <c r="E64" s="46"/>
+      <c r="F64" s="46"/>
+      <c r="G64" s="46"/>
+      <c r="H64" s="46"/>
+      <c r="I64" s="46"/>
+      <c r="J64" s="46"/>
+      <c r="K64" s="46"/>
+      <c r="L64" s="46"/>
+      <c r="M64" s="46"/>
+    </row>
+    <row r="65" spans="1:13" s="13" customFormat="1" ht="8.25" customHeight="1">
+      <c r="B65" s="14"/>
+      <c r="C65" s="14"/>
+      <c r="D65" s="14"/>
+      <c r="E65" s="18"/>
+      <c r="F65" s="18"/>
+      <c r="G65" s="16"/>
+      <c r="H65" s="16"/>
+      <c r="I65" s="16"/>
+      <c r="J65" s="18"/>
+      <c r="K65" s="18"/>
+      <c r="L65" s="18"/>
+    </row>
+    <row r="66" spans="1:13" s="21" customFormat="1" ht="8.25" customHeight="1">
+      <c r="A66" s="19"/>
+      <c r="B66" s="20"/>
+      <c r="C66" s="20"/>
+      <c r="D66" s="20"/>
+      <c r="E66" s="20"/>
+      <c r="F66" s="20"/>
+      <c r="G66" s="20"/>
+      <c r="H66" s="20"/>
+      <c r="I66" s="20"/>
+      <c r="J66" s="20"/>
+      <c r="K66" s="19"/>
+      <c r="L66" s="19"/>
+      <c r="M66" s="19"/>
+    </row>
+    <row r="67" spans="1:13" s="21" customFormat="1" ht="8.25" customHeight="1">
+      <c r="B67" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="C62" s="22"/>
-      <c r="D62" s="22"/>
-      <c r="E62" s="22"/>
-      <c r="F62" s="22"/>
-      <c r="G62" s="22"/>
-      <c r="H62" s="22"/>
-      <c r="I62" s="22"/>
-      <c r="J62" s="22"/>
-    </row>
-    <row r="63" spans="1:13" ht="8.25" customHeight="1"/>
-    <row r="64" spans="1:13" ht="8.25" customHeight="1">
-      <c r="B64" s="22" t="s">
+      <c r="C67" s="22"/>
+      <c r="D67" s="22"/>
+      <c r="E67" s="22"/>
+      <c r="F67" s="22"/>
+      <c r="G67" s="22"/>
+      <c r="H67" s="22"/>
+      <c r="I67" s="22"/>
+      <c r="J67" s="22"/>
+    </row>
+    <row r="68" spans="1:13" ht="8.25" customHeight="1"/>
+    <row r="69" spans="1:13" ht="8.25" customHeight="1">
+      <c r="B69" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="C64" s="22"/>
-      <c r="D64" s="22"/>
-    </row>
-    <row r="65" spans="2:4" ht="8.25" customHeight="1">
-      <c r="B65" s="22" t="s">
+      <c r="C69" s="22"/>
+      <c r="D69" s="22"/>
+    </row>
+    <row r="70" spans="1:13" ht="8.25" customHeight="1">
+      <c r="B70" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="C65" s="22"/>
-      <c r="D65" s="22"/>
-    </row>
-    <row r="66" spans="2:4" ht="8.25" customHeight="1">
-      <c r="B66" s="22" t="s">
+      <c r="C70" s="22"/>
+      <c r="D70" s="22"/>
+    </row>
+    <row r="71" spans="1:13" ht="8.25" customHeight="1">
+      <c r="B71" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="C66" s="22"/>
-      <c r="D66" s="22"/>
-    </row>
-    <row r="67" spans="2:4" ht="8.25" customHeight="1">
-      <c r="B67" s="23" t="s">
+      <c r="C71" s="22"/>
+      <c r="D71" s="22"/>
+    </row>
+    <row r="72" spans="1:13" ht="8.25" customHeight="1">
+      <c r="B72" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="C67" s="23"/>
-      <c r="D67" s="23"/>
+      <c r="C72" s="23"/>
+      <c r="D72" s="23"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="8">
+    <mergeCell ref="B61:M61"/>
+    <mergeCell ref="B62:M62"/>
+    <mergeCell ref="B63:M63"/>
     <mergeCell ref="B6:B9"/>
     <mergeCell ref="C6:C9"/>
     <mergeCell ref="E6:J6"/>
@@ -2367,7 +2468,8 @@
     <mergeCell ref="G7:J7"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B67" r:id="rId1" xr:uid="{4C8609E4-FC82-4503-A992-D1D629E0B105}"/>
+    <hyperlink ref="B72" r:id="rId1" xr:uid="{4C8609E4-FC82-4503-A992-D1D629E0B105}"/>
+    <hyperlink ref="B64" r:id="rId2" xr:uid="{01756EB4-57D4-4B8C-A40E-3589528D1D1B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Deploying to gh-pages from  @ 61c1d5f582bba1aa8dfa968773bd571ec5bb7b8d 🚀
</commit_message>
<xml_diff>
--- a/assets/excel/2026_4-1-5.xlsx
+++ b/assets/excel/2026_4-1-5.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Hannover\Dez15_Uebergreifende_Analysen\Projekte\Integrationsmonitoring\Schlesier\MT_Site\assets\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BiesterChristophLSN\Desktop\MZ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D43729AF-4BCB-484D-BE29-F6A5FD35611F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{81A6BD7D-24BF-4F2A-B887-24FB8A233B22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{25B46B2B-FF1A-413B-AD77-D797683F7C16}"/>
+    <workbookView xWindow="20052" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{25B46B2B-FF1A-413B-AD77-D797683F7C16}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="33">
   <si>
     <t>Indikator 4.1.5: Frühe Schulabgänger/-innen und Personen mit niedrigem Bildungsstand nach Migrationsstatus und Geschlecht</t>
   </si>
@@ -131,6 +131,18 @@
   </si>
   <si>
     <t>Migration und Teilhabe - Integrationsmonitoring Niedersachsen 2026</t>
+  </si>
+  <si>
+    <t>https://www.destatis.de/DE/Themen/Gesellschaft-Umwelt/Bevoelkerung/Haushalte-Familien/Methoden/mikrozensus-2020.html</t>
+  </si>
+  <si>
+    <t>3)  Ab der Veröffentlichung der Endergebnisse 2023 und der Erstergebnisse 2024 werden für die Hochrechnung des Mikrozensus Daten der Bevölkerungsfortschreibung herangezogen, die auf den Eckwerten des Zensus 2022 basieren. Die Hochrechnung für die Jahre vor 2011 sowie für bislang veröffentlichte Ergebnisse des Mikrozensus 2011-2013 basiert auf den fortgeschriebenen Ergebnissen der Volkszählung 1987. In 2016 erfolgte die Umstellung auf eine neue Mikrozensus-Stichprobe (auf Basis des Zensus 2011). Ab 2017 wird nur noch die Bevölkerung in Privathaushalten (ohne Gemeinschaftsunterkünfte) ausgewiesen. Dadurch ergibt sich jeweils eine eingeschränkte Vergleichbarkeit mit den Vorjahren.</t>
+  </si>
+  <si>
+    <t>4) Seit dem Jahr 2018 wird im Mikrozensus der Migrationshintergrund im weiteren Sinne jährlich berichtet. Die in der Tabelle ab dem Jahr 2018 abgebildeten Daten zum Migrationshintergrund entsprechen dem Migrationshintergrund im weiteren Sinne, bis 2017 wird der Migrationshintergrund im engeren Sinne abgebildet. Die Vergleichbarkeit ist dadurch eingeschränkt.</t>
+  </si>
+  <si>
+    <t>5) Die Ergebnisse des Mikrozensus 2020 sind unter anderem aufgrund methodischer Effekte im Rahmen einer Neugestaltung der Erhebung sowie insbesondere aufgrund der Folgen der Corona-Pandemie in Ihrer Datenqualität eingeschränkt. Auf die Verwendung dieser Ergebnisse wird daher verzichtet. Weitere Informationen zur methodischen Neugestaltung des Mikrozensus ab 2020 und zu den Auswirkungen der Neugestaltung und der Corona-Krise auf die Ergebnisse des Jahres 2020 finden Sie auf der Informationsseite des Statistischen Bundesamtes:</t>
   </si>
 </sst>
 </file>
@@ -362,7 +374,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
@@ -471,6 +483,15 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -493,9 +514,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -533,7 +554,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -639,7 +660,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -781,7 +802,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -790,7 +811,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D08CA7DC-4AB7-41CE-9601-7AD578505D24}">
   <sheetPr codeName="Tabelle1"/>
-  <dimension ref="A1:M67"/>
+  <dimension ref="A1:M72"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.85546875" customWidth="1"/>
@@ -2301,65 +2322,145 @@
       <c r="K60" s="18"/>
       <c r="L60" s="18"/>
     </row>
-    <row r="61" spans="1:13" s="21" customFormat="1" ht="8.25" customHeight="1">
-      <c r="A61" s="19"/>
-      <c r="B61" s="20"/>
-      <c r="C61" s="20"/>
-      <c r="D61" s="20"/>
-      <c r="E61" s="20"/>
-      <c r="F61" s="20"/>
-      <c r="G61" s="20"/>
-      <c r="H61" s="20"/>
-      <c r="I61" s="20"/>
-      <c r="J61" s="20"/>
-      <c r="K61" s="19"/>
-      <c r="L61" s="19"/>
-      <c r="M61" s="19"/>
-    </row>
-    <row r="62" spans="1:13" s="21" customFormat="1" ht="8.25" customHeight="1">
-      <c r="B62" s="22" t="s">
+    <row r="61" spans="1:13" s="13" customFormat="1" ht="26.25" customHeight="1">
+      <c r="B61" s="44" t="s">
+        <v>30</v>
+      </c>
+      <c r="C61" s="44"/>
+      <c r="D61" s="44"/>
+      <c r="E61" s="44"/>
+      <c r="F61" s="44"/>
+      <c r="G61" s="44"/>
+      <c r="H61" s="44"/>
+      <c r="I61" s="44"/>
+      <c r="J61" s="44"/>
+      <c r="K61" s="44"/>
+      <c r="L61" s="44"/>
+      <c r="M61" s="44"/>
+    </row>
+    <row r="62" spans="1:13" s="13" customFormat="1" ht="20.25" customHeight="1">
+      <c r="B62" s="44" t="s">
+        <v>31</v>
+      </c>
+      <c r="C62" s="44"/>
+      <c r="D62" s="44"/>
+      <c r="E62" s="44"/>
+      <c r="F62" s="44"/>
+      <c r="G62" s="44"/>
+      <c r="H62" s="44"/>
+      <c r="I62" s="44"/>
+      <c r="J62" s="44"/>
+      <c r="K62" s="44"/>
+      <c r="L62" s="44"/>
+      <c r="M62" s="44"/>
+    </row>
+    <row r="63" spans="1:13" s="13" customFormat="1" ht="24" customHeight="1">
+      <c r="B63" s="44" t="s">
+        <v>32</v>
+      </c>
+      <c r="C63" s="44"/>
+      <c r="D63" s="44"/>
+      <c r="E63" s="44"/>
+      <c r="F63" s="44"/>
+      <c r="G63" s="44"/>
+      <c r="H63" s="44"/>
+      <c r="I63" s="44"/>
+      <c r="J63" s="44"/>
+      <c r="K63" s="44"/>
+      <c r="L63" s="44"/>
+      <c r="M63" s="44"/>
+    </row>
+    <row r="64" spans="1:13" s="13" customFormat="1" ht="8.25" customHeight="1">
+      <c r="B64" s="45" t="s">
+        <v>29</v>
+      </c>
+      <c r="C64" s="46"/>
+      <c r="D64" s="46"/>
+      <c r="E64" s="46"/>
+      <c r="F64" s="46"/>
+      <c r="G64" s="46"/>
+      <c r="H64" s="46"/>
+      <c r="I64" s="46"/>
+      <c r="J64" s="46"/>
+      <c r="K64" s="46"/>
+      <c r="L64" s="46"/>
+      <c r="M64" s="46"/>
+    </row>
+    <row r="65" spans="1:13" s="13" customFormat="1" ht="8.25" customHeight="1">
+      <c r="B65" s="14"/>
+      <c r="C65" s="14"/>
+      <c r="D65" s="14"/>
+      <c r="E65" s="18"/>
+      <c r="F65" s="18"/>
+      <c r="G65" s="16"/>
+      <c r="H65" s="16"/>
+      <c r="I65" s="16"/>
+      <c r="J65" s="18"/>
+      <c r="K65" s="18"/>
+      <c r="L65" s="18"/>
+    </row>
+    <row r="66" spans="1:13" s="21" customFormat="1" ht="8.25" customHeight="1">
+      <c r="A66" s="19"/>
+      <c r="B66" s="20"/>
+      <c r="C66" s="20"/>
+      <c r="D66" s="20"/>
+      <c r="E66" s="20"/>
+      <c r="F66" s="20"/>
+      <c r="G66" s="20"/>
+      <c r="H66" s="20"/>
+      <c r="I66" s="20"/>
+      <c r="J66" s="20"/>
+      <c r="K66" s="19"/>
+      <c r="L66" s="19"/>
+      <c r="M66" s="19"/>
+    </row>
+    <row r="67" spans="1:13" s="21" customFormat="1" ht="8.25" customHeight="1">
+      <c r="B67" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="C62" s="22"/>
-      <c r="D62" s="22"/>
-      <c r="E62" s="22"/>
-      <c r="F62" s="22"/>
-      <c r="G62" s="22"/>
-      <c r="H62" s="22"/>
-      <c r="I62" s="22"/>
-      <c r="J62" s="22"/>
-    </row>
-    <row r="63" spans="1:13" ht="8.25" customHeight="1"/>
-    <row r="64" spans="1:13" ht="8.25" customHeight="1">
-      <c r="B64" s="22" t="s">
+      <c r="C67" s="22"/>
+      <c r="D67" s="22"/>
+      <c r="E67" s="22"/>
+      <c r="F67" s="22"/>
+      <c r="G67" s="22"/>
+      <c r="H67" s="22"/>
+      <c r="I67" s="22"/>
+      <c r="J67" s="22"/>
+    </row>
+    <row r="68" spans="1:13" ht="8.25" customHeight="1"/>
+    <row r="69" spans="1:13" ht="8.25" customHeight="1">
+      <c r="B69" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="C64" s="22"/>
-      <c r="D64" s="22"/>
-    </row>
-    <row r="65" spans="2:4" ht="8.25" customHeight="1">
-      <c r="B65" s="22" t="s">
+      <c r="C69" s="22"/>
+      <c r="D69" s="22"/>
+    </row>
+    <row r="70" spans="1:13" ht="8.25" customHeight="1">
+      <c r="B70" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="C65" s="22"/>
-      <c r="D65" s="22"/>
-    </row>
-    <row r="66" spans="2:4" ht="8.25" customHeight="1">
-      <c r="B66" s="22" t="s">
+      <c r="C70" s="22"/>
+      <c r="D70" s="22"/>
+    </row>
+    <row r="71" spans="1:13" ht="8.25" customHeight="1">
+      <c r="B71" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="C66" s="22"/>
-      <c r="D66" s="22"/>
-    </row>
-    <row r="67" spans="2:4" ht="8.25" customHeight="1">
-      <c r="B67" s="23" t="s">
+      <c r="C71" s="22"/>
+      <c r="D71" s="22"/>
+    </row>
+    <row r="72" spans="1:13" ht="8.25" customHeight="1">
+      <c r="B72" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="C67" s="23"/>
-      <c r="D67" s="23"/>
+      <c r="C72" s="23"/>
+      <c r="D72" s="23"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="8">
+    <mergeCell ref="B61:M61"/>
+    <mergeCell ref="B62:M62"/>
+    <mergeCell ref="B63:M63"/>
     <mergeCell ref="B6:B9"/>
     <mergeCell ref="C6:C9"/>
     <mergeCell ref="E6:J6"/>
@@ -2367,7 +2468,8 @@
     <mergeCell ref="G7:J7"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B67" r:id="rId1" xr:uid="{4C8609E4-FC82-4503-A992-D1D629E0B105}"/>
+    <hyperlink ref="B72" r:id="rId1" xr:uid="{4C8609E4-FC82-4503-A992-D1D629E0B105}"/>
+    <hyperlink ref="B64" r:id="rId2" xr:uid="{01756EB4-57D4-4B8C-A40E-3589528D1D1B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>